<commit_message>
Dessa vez é a 1º versão que aparenta ser infalível para teste,com botão de baixar planilha e imprimir etiquetas, com uma tela de carregamento funcional e todo o programa organizado
</commit_message>
<xml_diff>
--- a/modelos/Modelo_Etiqueta_Luari.xlsx
+++ b/modelos/Modelo_Etiqueta_Luari.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/484c53c37b433491/Desktop/Projetos/Transformers - Convertedor de arquivos/modelos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="177" documentId="13_ncr:1_{3AD2A3B6-EB1E-4204-BED8-0676429C1447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5576A705-831B-49C9-AC13-2AD3D137909E}"/>
+  <xr:revisionPtr revIDLastSave="212" documentId="13_ncr:1_{3AD2A3B6-EB1E-4204-BED8-0676429C1447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{018C28C8-6274-493A-BAA5-4074FA949D6B}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -332,7 +332,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -366,7 +366,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -458,13 +457,13 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>513523</xdr:colOff>
+      <xdr:colOff>741194</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>41414</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>1904688</xdr:colOff>
+      <xdr:colOff>2132359</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>300464</xdr:rowOff>
     </xdr:to>
@@ -495,8 +494,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="513523" y="231914"/>
-          <a:ext cx="2153478" cy="830550"/>
+          <a:off x="741194" y="375951"/>
+          <a:ext cx="2153165" cy="830550"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -508,15 +507,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>19708</xdr:colOff>
+      <xdr:colOff>46378</xdr:colOff>
       <xdr:row>27</xdr:row>
-      <xdr:rowOff>49696</xdr:rowOff>
+      <xdr:rowOff>45886</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>715926</xdr:colOff>
+      <xdr:colOff>742596</xdr:colOff>
       <xdr:row>30</xdr:row>
-      <xdr:rowOff>173934</xdr:rowOff>
+      <xdr:rowOff>170124</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -545,7 +544,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="19708" y="5810679"/>
+          <a:off x="46378" y="5920906"/>
           <a:ext cx="696218" cy="695738"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1007,7 +1006,7 @@
     <col min="2" max="2" width="47.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3"/>
       <c r="B1" s="3"/>
     </row>
@@ -1053,63 +1052,63 @@
     </row>
     <row r="10" spans="1:2" ht="1.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="12"/>
-      <c r="B10" s="13"/>
+      <c r="B10" s="12"/>
     </row>
     <row r="11" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="12"/>
-      <c r="B11" s="13"/>
+      <c r="B11" s="12"/>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="13"/>
-      <c r="B12" s="13"/>
+      <c r="A12" s="12"/>
+      <c r="B12" s="12"/>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="13"/>
-      <c r="B13" s="13"/>
+      <c r="A13" s="12"/>
+      <c r="B13" s="12"/>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="13"/>
-      <c r="B14" s="13"/>
+      <c r="A14" s="12"/>
+      <c r="B14" s="12"/>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="13"/>
-      <c r="B15" s="13"/>
+      <c r="A15" s="12"/>
+      <c r="B15" s="12"/>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="13"/>
-      <c r="B16" s="13"/>
+      <c r="A16" s="12"/>
+      <c r="B16" s="12"/>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="13"/>
-      <c r="B17" s="13"/>
+      <c r="A17" s="12"/>
+      <c r="B17" s="12"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="13"/>
-      <c r="B18" s="13"/>
+      <c r="A18" s="12"/>
+      <c r="B18" s="12"/>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="13"/>
-      <c r="B19" s="13"/>
+      <c r="A19" s="12"/>
+      <c r="B19" s="12"/>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="13"/>
-      <c r="B20" s="13"/>
+      <c r="A20" s="12"/>
+      <c r="B20" s="12"/>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="13"/>
-      <c r="B21" s="13"/>
+      <c r="A21" s="12"/>
+      <c r="B21" s="12"/>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="13"/>
-      <c r="B22" s="13"/>
+      <c r="A22" s="12"/>
+      <c r="B22" s="12"/>
     </row>
     <row r="23" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="13"/>
-      <c r="B23" s="13"/>
+      <c r="A23" s="12"/>
+      <c r="B23" s="12"/>
     </row>
     <row r="24" spans="1:2" ht="1.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="13"/>
-      <c r="B24" s="13"/>
+      <c r="A24" s="12"/>
+      <c r="B24" s="12"/>
     </row>
     <row r="25" spans="1:2" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
@@ -1128,22 +1127,22 @@
       <c r="B27" s="7"/>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" s="17"/>
-      <c r="B28" s="14" t="s">
+      <c r="A28" s="16"/>
+      <c r="B28" s="13" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" s="18"/>
-      <c r="B29" s="15"/>
+      <c r="A29" s="17"/>
+      <c r="B29" s="14"/>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" s="18"/>
-      <c r="B30" s="15"/>
+      <c r="A30" s="17"/>
+      <c r="B30" s="14"/>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" s="19"/>
-      <c r="B31" s="16"/>
+      <c r="A31" s="18"/>
+      <c r="B31" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1158,7 +1157,7 @@
     <hyperlink ref="A27" r:id="rId1" xr:uid="{D484840B-E6BA-45D8-A37A-CD7AD525D4C0}"/>
   </hyperlinks>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <pageSetup paperSize="260" scale="93" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId2"/>
+  <pageSetup paperSize="259" scale="45" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId2"/>
   <drawing r:id="rId3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Chegou a impressora nova então consegui relizar a impresão normalmente e arrumei a estrtura da etiqueta para que ela ficasse com o qrcode com a tela cheia dele
</commit_message>
<xml_diff>
--- a/modelos/Modelo_Etiqueta_Luari.xlsx
+++ b/modelos/Modelo_Etiqueta_Luari.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/484c53c37b433491/Desktop/Projetos/Transformers - Convertedor de arquivos/modelos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="212" documentId="13_ncr:1_{3AD2A3B6-EB1E-4204-BED8-0676429C1447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{018C28C8-6274-493A-BAA5-4074FA949D6B}"/>
+  <xr:revisionPtr revIDLastSave="273" documentId="13_ncr:1_{3AD2A3B6-EB1E-4204-BED8-0676429C1447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7CE59BF8-85F3-4F06-AEA1-AB4FFB8874D5}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,14 +17,14 @@
     <sheet name="Config" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Etiqueta!$A$1:$B$31</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Etiqueta!$A$1:$C$31</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="33">
   <si>
     <t>Data:</t>
   </si>
@@ -116,28 +116,20 @@
     <t>Operador:</t>
   </si>
   <si>
-    <t>www.luariembalagens.com.br</t>
-  </si>
-  <si>
-    <t>Se possuir alguma solicitação ou sugestão com relação à
-montagem dos pallets, favor enviar e-mail para:
-contato@luariembalagens.com.br</t>
-  </si>
-  <si>
     <t>OdP:</t>
   </si>
   <si>
     <t>Máquina:</t>
   </si>
   <si>
-    <t xml:space="preserve">Pesquisa de Qualidade: </t>
+    <t>Cliente:</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -168,14 +160,6 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -197,7 +181,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -209,76 +193,6 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -311,28 +225,16 @@
         <color indexed="64"/>
       </right>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -342,51 +244,15 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -406,13 +272,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>0</xdr:col>
+      <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>2</xdr:col>
       <xdr:colOff>3108077</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -456,13 +322,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>0</xdr:col>
+      <xdr:col>1</xdr:col>
       <xdr:colOff>741194</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>41414</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>2</xdr:col>
       <xdr:colOff>2132359</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>300464</xdr:rowOff>
@@ -496,206 +362,6 @@
         <a:xfrm>
           <a:off x="741194" y="375951"/>
           <a:ext cx="2153165" cy="830550"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>46378</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>45886</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>742596</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>170124</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Imagem 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F0DF434E-ADAE-C493-D53E-09A2C1108185}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="46378" y="5920906"/>
-          <a:ext cx="696218" cy="695738"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>1386941</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>57563</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>1722529</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>12151</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="13" name="Gráfico 12" descr="Contorno de rosto irritado com preenchimento sólido">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F9952094-FF4B-182B-D179-BED0B3C12EDD}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4">
-          <a:extLst>
-            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
-              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId5"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2369748" y="6015018"/>
-          <a:ext cx="335588" cy="335588"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>1914809</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>46292</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>2259730</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>10213</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="15" name="Gráfico 14" descr="Contorno de rosto nervoso com preenchimento sólido">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{34BD4FAE-DFFE-0C1F-A82B-D88B8ADCD25E}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6">
-          <a:extLst>
-            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
-              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId7"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2897616" y="6003747"/>
-          <a:ext cx="344921" cy="344921"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>2440280</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>47291</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>2794043</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>20054</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="17" name="Gráfico 16" descr="Contorno de rosto divertido com preenchimento sólido">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1D25D3F5-0AE5-392F-7210-70A6E823A351}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8">
-          <a:extLst>
-            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
-              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId9"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3423087" y="6004746"/>
-          <a:ext cx="353763" cy="353763"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -999,166 +665,191 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" customWidth="1"/>
-    <col min="2" max="2" width="47.28515625" customWidth="1"/>
+    <col min="1" max="1" width="0.42578125" customWidth="1"/>
+    <col min="2" max="2" width="11.42578125" customWidth="1"/>
+    <col min="3" max="3" width="46.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3"/>
+    <row r="1" spans="1:3" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="3"/>
-    </row>
-    <row r="2" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="5"/>
-      <c r="B2" s="5"/>
-    </row>
-    <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="5"/>
-      <c r="B3" s="5"/>
-    </row>
-    <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5"/>
-    </row>
-    <row r="5" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5"/>
-    </row>
-    <row r="6" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C1" s="3"/>
+    </row>
+    <row r="2" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="6"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+    </row>
+    <row r="3" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="6"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+    </row>
+    <row r="4" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="6"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+    </row>
+    <row r="5" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="6"/>
+      <c r="B5" s="6"/>
+      <c r="C5" s="6"/>
+    </row>
+    <row r="6" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="B6" s="2"/>
-    </row>
-    <row r="7" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+      <c r="B6" s="4"/>
+      <c r="C6" s="7"/>
+    </row>
+    <row r="7" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="2"/>
-    </row>
-    <row r="8" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="4"/>
+      <c r="C7" s="2"/>
+    </row>
+    <row r="8" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B8" s="2"/>
-    </row>
-    <row r="9" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+      <c r="B8" s="4"/>
+      <c r="C8" s="2"/>
+    </row>
+    <row r="9" spans="1:3" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B9" s="2"/>
-    </row>
-    <row r="10" spans="1:2" ht="1.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="12"/>
-      <c r="B10" s="12"/>
-    </row>
-    <row r="11" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="12"/>
-      <c r="B11" s="12"/>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="12"/>
-      <c r="B12" s="12"/>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="12"/>
-      <c r="B13" s="12"/>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="12"/>
-      <c r="B14" s="12"/>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="12"/>
-      <c r="B15" s="12"/>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="12"/>
-      <c r="B16" s="12"/>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="12"/>
-      <c r="B17" s="12"/>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="12"/>
-      <c r="B18" s="12"/>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="12"/>
-      <c r="B19" s="12"/>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="12"/>
-      <c r="B20" s="12"/>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="12"/>
-      <c r="B21" s="12"/>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="12"/>
-      <c r="B22" s="12"/>
-    </row>
-    <row r="23" spans="1:2" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="12"/>
-      <c r="B23" s="12"/>
-    </row>
-    <row r="24" spans="1:2" ht="1.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="12"/>
-      <c r="B24" s="12"/>
-    </row>
-    <row r="25" spans="1:2" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="B25" s="9"/>
-    </row>
-    <row r="26" spans="1:2" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="10"/>
-      <c r="B26" s="11"/>
-    </row>
-    <row r="27" spans="1:2" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="B27" s="7"/>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" s="16"/>
-      <c r="B28" s="13" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" s="17"/>
-      <c r="B29" s="14"/>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" s="17"/>
-      <c r="B30" s="14"/>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" s="18"/>
-      <c r="B31" s="15"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="2"/>
+    </row>
+    <row r="10" spans="1:3" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="4"/>
+      <c r="C10" s="5"/>
+    </row>
+    <row r="11" spans="1:3" ht="2.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="6"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="6"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="6"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="6"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="6"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="6"/>
+      <c r="B17" s="6"/>
+      <c r="C17" s="6"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="6"/>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="6"/>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="6"/>
+      <c r="B20" s="6"/>
+      <c r="C20" s="6"/>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="6"/>
+      <c r="B21" s="6"/>
+      <c r="C21" s="6"/>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="6"/>
+      <c r="B22" s="6"/>
+      <c r="C22" s="6"/>
+    </row>
+    <row r="23" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="6"/>
+      <c r="B23" s="6"/>
+      <c r="C23" s="6"/>
+    </row>
+    <row r="24" spans="1:3" ht="1.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="6"/>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+    </row>
+    <row r="25" spans="1:3" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="6"/>
+      <c r="B25" s="6"/>
+      <c r="C25" s="6"/>
+    </row>
+    <row r="26" spans="1:3" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="6"/>
+      <c r="B26" s="6"/>
+      <c r="C26" s="6"/>
+    </row>
+    <row r="27" spans="1:3" ht="1.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="6"/>
+      <c r="B27" s="6"/>
+      <c r="C27" s="6"/>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="6"/>
+      <c r="B28" s="6"/>
+      <c r="C28" s="6"/>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="6"/>
+      <c r="B29" s="6"/>
+      <c r="C29" s="6"/>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="6"/>
+      <c r="B30" s="6"/>
+      <c r="C30" s="6"/>
+    </row>
+    <row r="31" spans="1:3" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="6"/>
+      <c r="B31" s="6"/>
+      <c r="C31" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A2:B5"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A25:B26"/>
-    <mergeCell ref="A10:B24"/>
-    <mergeCell ref="B28:B31"/>
-    <mergeCell ref="A28:A31"/>
+  <mergeCells count="7">
+    <mergeCell ref="A2:C5"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A11:C31"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink ref="A27" r:id="rId1" xr:uid="{D484840B-E6BA-45D8-A37A-CD7AD525D4C0}"/>
-  </hyperlinks>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <pageSetup paperSize="259" scale="45" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId2"/>
-  <drawing r:id="rId3"/>
+  <pageSetup paperSize="260" scale="88" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Comecei a fazer as 1º implantações do botão de imprimir, no caso estou vendo de transformar em PDF
</commit_message>
<xml_diff>
--- a/modelos/Modelo_Etiqueta_Luari.xlsx
+++ b/modelos/Modelo_Etiqueta_Luari.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/484c53c37b433491/Desktop/Projetos/Transformers - Convertedor de arquivos/modelos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="273" documentId="13_ncr:1_{3AD2A3B6-EB1E-4204-BED8-0676429C1447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7CE59BF8-85F3-4F06-AEA1-AB4FFB8874D5}"/>
+  <xr:revisionPtr revIDLastSave="277" documentId="13_ncr:1_{3AD2A3B6-EB1E-4204-BED8-0676429C1447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B1F32889-38BB-45B9-8B79-8427AB29A496}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -241,16 +241,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -270,56 +270,6 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>3108077</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Imagem 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{04972E56-C069-E084-1FC4-4D8B5B313B56}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm flipV="1">
-          <a:off x="0" y="0"/>
-          <a:ext cx="3875314" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
@@ -347,7 +297,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -371,10 +321,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -698,39 +644,39 @@
       <c r="C5" s="6"/>
     </row>
     <row r="6" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B6" s="4"/>
-      <c r="C6" s="7"/>
+      <c r="B6" s="7"/>
+      <c r="C6" s="5"/>
     </row>
     <row r="7" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="4"/>
+      <c r="B7" s="7"/>
       <c r="C7" s="2"/>
     </row>
     <row r="8" spans="1:3" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B8" s="4"/>
+      <c r="B8" s="7"/>
       <c r="C8" s="2"/>
     </row>
     <row r="9" spans="1:3" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B9" s="4"/>
+      <c r="B9" s="7"/>
       <c r="C9" s="2"/>
     </row>
     <row r="10" spans="1:3" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B10" s="4"/>
-      <c r="C10" s="5"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="4"/>
     </row>
     <row r="11" spans="1:3" ht="2.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6"/>
@@ -839,13 +785,13 @@
     </row>
   </sheetData>
   <mergeCells count="7">
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A11:C31"/>
     <mergeCell ref="A2:C5"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A11:C31"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
   <pageSetup paperSize="260" scale="88" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>

</xml_diff>